<commit_message>
Update Emerging Compounder Radar
</commit_message>
<xml_diff>
--- a/data/compounder_radar.xlsx
+++ b/data/compounder_radar.xlsx
@@ -426,16 +426,16 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="23" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
     <col width="45" customWidth="1" min="15" max="15"/>
     <col width="19" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
   </cols>
@@ -545,19 +545,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Micron Technology, Inc.</t>
+          <t>Arista Networks, Inc.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>81.3</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -565,27 +565,29 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.06713489726936261</v>
+        <v>0.2714652572159764</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.006929629272242499</v>
+        <v>0.3708447402164197</v>
       </c>
       <c r="H2" t="n">
-        <v>0.7256899999999999</v>
+        <v>0.63004</v>
       </c>
       <c r="I2" t="n">
-        <v>0.3487</v>
+        <v>0.14119</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8351558770343581</v>
+        <v>0.2648009752477871</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.8728631705846895</v>
+        <v>-0.3930142576986272</v>
       </c>
       <c r="L2" t="n">
-        <v>0.9568004530136458</v>
-      </c>
-      <c r="M2" t="inlineStr"/>
+        <v>0.6737693863789616</v>
+      </c>
+      <c r="M2" t="n">
+        <v>237955268608</v>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
           <t>High</t>
@@ -593,43 +595,43 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Høj bruttomargin, positivt momentum, analytiker-upside over 20 %</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q2" t="b">
         <v>1</v>
       </c>
       <c r="R2" t="n">
-        <v>0.5916866288645946</v>
+        <v>0.3310052780877977</v>
       </c>
       <c r="S2" t="n">
-        <v>0.8896770801335447</v>
+        <v>0.4663091696109241</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Advanced Micro Devices, Inc.</t>
+          <t>NVIDIA Corporation</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>79.90000000000001</v>
+        <v>81.2</v>
       </c>
       <c r="D3" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -637,30 +639,32 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.1364359933536843</v>
+        <v>1.000450949944396</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4666355102918431</v>
+        <v>2.04239508347386</v>
       </c>
       <c r="H3" t="n">
-        <v>0.5306</v>
+        <v>0.74144995</v>
       </c>
       <c r="I3" t="n">
-        <v>0.03647</v>
+        <v>0.52727</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1949207659293497</v>
+        <v>0.3521502946954813</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.6921013535820403</v>
+        <v>-0.2674138238971245</v>
       </c>
       <c r="L3" t="n">
-        <v>0.2816361576530917</v>
-      </c>
-      <c r="M3" t="inlineStr"/>
+        <v>1.316873935548505</v>
+      </c>
+      <c r="M3" t="n">
+        <v>5424535306240</v>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -669,39 +673,39 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q3" t="b">
         <v>1</v>
       </c>
       <c r="R3" t="n">
-        <v>0.3431972891016541</v>
+        <v>0.06014672155350387</v>
       </c>
       <c r="S3" t="n">
-        <v>0.8881354894345377</v>
+        <v>0.3045914419713429</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Eli Lilly and Company</t>
+          <t>Micron Technology, Inc.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>76.90000000000001</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -709,27 +713,29 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.3168737488062043</v>
+        <v>0.06713489726936261</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5171329563234539</v>
+        <v>-0.006929629272242499</v>
       </c>
       <c r="H4" t="n">
-        <v>0.8283199999999999</v>
+        <v>0.7256899999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>0.20739001</v>
+        <v>0.3487</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1387614147107084</v>
+        <v>0.7115178276376812</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.4437290433045588</v>
+        <v>-0.8707111683398475</v>
       </c>
       <c r="L4" t="n">
-        <v>0.3127165480927688</v>
-      </c>
-      <c r="M4" t="inlineStr"/>
+        <v>0.8171686013793824</v>
+      </c>
+      <c r="M4" t="n">
+        <v>991121571840</v>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
           <t>High</t>
@@ -737,43 +743,43 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
+          <t>Høj bruttomargin, positivt momentum, analytiker-upside over 20 %</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q4" t="b">
         <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>0.2313477828196622</v>
+        <v>0.3573526703199177</v>
       </c>
       <c r="S4" t="n">
-        <v>0.1255671610267297</v>
+        <v>1.293279161436129</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fortinet, Inc.</t>
+          <t>Advanced Micro Devices, Inc.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>76.8</v>
+        <v>76</v>
       </c>
       <c r="D5" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -781,28 +787,28 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.1546194776009138</v>
+        <v>0.1364359933536843</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3167495145145989</v>
+        <v>0.4666355102918431</v>
       </c>
       <c r="H5" t="n">
-        <v>0.80204004</v>
+        <v>0.55724</v>
       </c>
       <c r="I5" t="n">
-        <v>0.14166</v>
+        <v>0.05128</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.02264873475889961</v>
+        <v>0.2688985435286328</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.5703694626554745</v>
+        <v>-0.6912859980139027</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.03970888387581917</v>
+        <v>0.3889830609923983</v>
       </c>
       <c r="M5" t="n">
-        <v>119749410816</v>
+        <v>789073100800</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -821,60 +827,62 @@
         <v>1</v>
       </c>
       <c r="R5" t="n">
-        <v>0.9208872214198582</v>
+        <v>0.1833716776756134</v>
       </c>
       <c r="S5" t="n">
-        <v>0.9868726868338145</v>
+        <v>1.51096096286526</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sandisk Corporation</t>
+          <t>Fortinet, Inc.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>74.5</v>
+        <v>75.5</v>
       </c>
       <c r="D6" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>High Conviction</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.09932312697218015</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
+        <v>0.1546194776009138</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.3167495145145989</v>
+      </c>
       <c r="H6" t="n">
-        <v>0.56038</v>
+        <v>0.80204004</v>
       </c>
       <c r="I6" t="n">
-        <v>0.22823</v>
+        <v>0.14166</v>
       </c>
       <c r="J6" t="n">
-        <v>0.7218331094772636</v>
+        <v>0.007672575795540038</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.9685333416147139</v>
+        <v>-0.5392758707090954</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7452847294589178</v>
+        <v>0.01422755256127322</v>
       </c>
       <c r="M6" t="n">
-        <v>190744051712</v>
+        <v>117130051584</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -883,43 +891,43 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Høj bruttomargin, positivt momentum, analytiker-upside over 20 %</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q6" t="b">
         <v>1</v>
       </c>
       <c r="R6" t="n">
-        <v>0.1079059427048485</v>
+        <v>0.4785588365728168</v>
       </c>
       <c r="S6" t="n">
-        <v>1.252605198502335</v>
+        <v>1.022551612471996</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Dell Technologies Inc.</t>
+          <t>Amphenol Corporation</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>70.7</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -927,28 +935,28 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.03534983888485344</v>
+        <v>0.2230660589034148</v>
       </c>
       <c r="G7" t="n">
-        <v>0.388859258627138</v>
+        <v>0.2972340671812952</v>
       </c>
       <c r="H7" t="n">
-        <v>0.19212</v>
+        <v>0.38952</v>
       </c>
       <c r="I7" t="n">
-        <v>0.07004000000000001</v>
+        <v>0.14473</v>
       </c>
       <c r="J7" t="n">
-        <v>0.1719328236445854</v>
+        <v>0.1706987823619812</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.743088900284369</v>
+        <v>-0.3810734129329708</v>
       </c>
       <c r="L7" t="n">
-        <v>0.2313758469259725</v>
+        <v>0.4479419885217928</v>
       </c>
       <c r="M7" t="n">
-        <v>277208006656</v>
+        <v>208596123648</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -957,7 +965,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Stærk eps-vækst, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, positivt momentum</t>
         </is>
       </c>
       <c r="P7" t="n">
@@ -967,33 +975,33 @@
         <v>1</v>
       </c>
       <c r="R7" t="n">
-        <v>0.9432393281153402</v>
+        <v>0.2401934174574814</v>
       </c>
       <c r="S7" t="n">
-        <v>2.437388951944431</v>
+        <v>0.3301740732320491</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Marvell Technology, Inc.</t>
+          <t>Broadcom Inc.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>70.5</v>
+        <v>74.8</v>
       </c>
       <c r="D8" t="n">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1001,71 +1009,73 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.1144958764235571</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
+        <v>0.2437842600004176</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.2159817111378917</v>
+      </c>
       <c r="H8" t="n">
-        <v>0.5150299699999999</v>
+        <v>0.76284</v>
       </c>
       <c r="I8" t="n">
-        <v>0.03808</v>
+        <v>0.121190004</v>
       </c>
       <c r="J8" t="n">
-        <v>0.3258376983615017</v>
+        <v>0.2340669066766412</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.6829312346793962</v>
+        <v>-0.3410557321862726</v>
       </c>
       <c r="L8" t="n">
-        <v>0.4771164091132353</v>
+        <v>0.686301048735349</v>
       </c>
       <c r="M8" t="n">
-        <v>173921665024</v>
+        <v>2035102646272</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q8" t="b">
         <v>1</v>
       </c>
       <c r="R8" t="n">
-        <v>0.1359749795783063</v>
+        <v>0.03848414109854015</v>
       </c>
       <c r="S8" t="n">
-        <v>1.307600188596483</v>
+        <v>0.3826792124922158</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Howmet Aerospace Inc.</t>
+          <t>Palantir Technologies Inc.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HWM</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>70.40000000000001</v>
+        <v>74.7</v>
       </c>
       <c r="D9" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1073,28 +1083,26 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.1337158522423005</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.495146138791156</v>
-      </c>
+        <v>0.3291712528765784</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>0.35046002</v>
+        <v>0.84796</v>
       </c>
       <c r="I9" t="n">
-        <v>0.11918</v>
+        <v>0.17292999</v>
       </c>
       <c r="J9" t="n">
-        <v>0.09285464832017887</v>
+        <v>0.1040184872972503</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.408220996018719</v>
+        <v>-0.3816057205976396</v>
       </c>
       <c r="L9" t="n">
-        <v>0.2274617161433828</v>
+        <v>0.2725810481413775</v>
       </c>
       <c r="M9" t="n">
-        <v>114566774784</v>
+        <v>413350068224</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -1103,43 +1111,43 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, positivt momentum</t>
+          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>100</v>
+        <v>88.88888888888889</v>
       </c>
       <c r="Q9" t="b">
         <v>1</v>
       </c>
       <c r="R9" t="n">
-        <v>0.1618842604945363</v>
+        <v>0.2550893154075689</v>
       </c>
       <c r="S9" t="n">
-        <v>0.3523480848477396</v>
+        <v>0.3230520865670188</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Interactive Brokers Group, Inc.</t>
+          <t>Booking Holdings Inc. Common St</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IBKR</t>
+          <t>BKNG</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>69.40000000000001</v>
+        <v>74</v>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1147,28 +1155,28 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.3459787421885367</v>
+        <v>0.1634869878187224</v>
       </c>
       <c r="G10" t="n">
-        <v>0.3328887406583814</v>
+        <v>0.2943673092572356</v>
       </c>
       <c r="H10" t="n">
-        <v>0.93036</v>
+        <v>0.87227994</v>
       </c>
       <c r="I10" t="n">
-        <v>0.022839999</v>
+        <v>0.2038</v>
       </c>
       <c r="J10" t="n">
-        <v>0.2189933903133903</v>
+        <v>0.1069914653483817</v>
       </c>
       <c r="K10" t="n">
-        <v>-0.3282051282051281</v>
+        <v>-0.2997854677735287</v>
       </c>
       <c r="L10" t="n">
-        <v>0.6672454861111111</v>
+        <v>0.3568934349719974</v>
       </c>
       <c r="M10" t="n">
-        <v>148843495424</v>
+        <v>166149439488</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -1187,33 +1195,33 @@
         <v>1</v>
       </c>
       <c r="R10" t="n">
-        <v>0.1079134997425473</v>
+        <v>0.2550153802075548</v>
       </c>
       <c r="S10" t="n">
-        <v>0.1653941636847271</v>
+        <v>0.2121822677669754</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>F5, Inc.</t>
+          <t>ServiceNow, Inc.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>69.3</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1221,37 +1229,37 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.04631913174341684</v>
+        <v>0.2237651786474262</v>
       </c>
       <c r="G11" t="n">
-        <v>0.3082491584064506</v>
+        <v>0.7345580184539504</v>
       </c>
       <c r="H11" t="n">
-        <v>0.8192700000000001</v>
+        <v>0.74768996</v>
       </c>
       <c r="I11" t="n">
-        <v>0.07995999600000001</v>
+        <v>0.04249</v>
       </c>
       <c r="J11" t="n">
-        <v>0.07321274763135222</v>
+        <v>0.1231007367072392</v>
       </c>
       <c r="K11" t="n">
-        <v>-0.4493417005044913</v>
+        <v>-0.3494554772581678</v>
       </c>
       <c r="L11" t="n">
-        <v>0.162933347938003</v>
+        <v>0.352264436296976</v>
       </c>
       <c r="M11" t="n">
-        <v>23091245056</v>
+        <v>129108688896</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Stærk eps-vækst, høj bruttomargin, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P11" t="n">
@@ -1261,33 +1269,33 @@
         <v>1</v>
       </c>
       <c r="R11" t="n">
-        <v>0.2428836520845277</v>
+        <v>0.3343306137395301</v>
       </c>
       <c r="S11" t="n">
-        <v>0.4248752665683944</v>
+        <v>0.2167982129538544</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Applied Materials, Inc.</t>
+          <t>DexCom, Inc.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>DXCM</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>68.8</v>
+        <v>72</v>
       </c>
       <c r="D12" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1295,28 +1303,28 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.03233470456886756</v>
+        <v>0.1701360960301399</v>
       </c>
       <c r="G12" t="n">
-        <v>0.05191743203490939</v>
+        <v>0.365979383233586</v>
       </c>
       <c r="H12" t="n">
-        <v>0.48956</v>
+        <v>0.62473</v>
       </c>
       <c r="I12" t="n">
-        <v>0.14858</v>
+        <v>0.103310004</v>
       </c>
       <c r="J12" t="n">
-        <v>0.211202350398487</v>
+        <v>0.1025368731563421</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.7019162115744583</v>
+        <v>-0.3615339233038348</v>
       </c>
       <c r="L12" t="n">
-        <v>0.3008939627206245</v>
+        <v>0.2836161879895558</v>
       </c>
       <c r="M12" t="n">
-        <v>411437727744</v>
+        <v>31981324288</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -1325,7 +1333,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Høj bruttomargin, positivt momentum, analytiker-upside over 20 %</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P12" t="n">
@@ -1335,33 +1343,33 @@
         <v>1</v>
       </c>
       <c r="R12" t="n">
-        <v>0.288501973340042</v>
+        <v>0.3913971468118593</v>
       </c>
       <c r="S12" t="n">
-        <v>0.4909915340075093</v>
+        <v>0.2126198417531036</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>United Airlines Holdings, Inc.</t>
+          <t>Microsoft Corporation</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>UAL</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>68.8</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1369,28 +1377,28 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.09529134601036815</v>
+        <v>0.1612397915820203</v>
       </c>
       <c r="G13" t="n">
-        <v>0.6599631084110487</v>
+        <v>0.2285599828574523</v>
       </c>
       <c r="H13" t="n">
-        <v>0.31816</v>
+        <v>0.67944</v>
       </c>
       <c r="I13" t="n">
-        <v>0.03381</v>
+        <v>0.14088</v>
       </c>
       <c r="J13" t="n">
-        <v>0.2629658073058649</v>
+        <v>0.1267206544130883</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.3407586260612196</v>
+        <v>-0.3015860317206345</v>
       </c>
       <c r="L13" t="n">
-        <v>0.7717069714285716</v>
+        <v>0.4201807812189138</v>
       </c>
       <c r="M13" t="n">
-        <v>41671507968</v>
+        <v>3712698548224</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -1399,7 +1407,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Stærk eps-vækst, positivt momentum, analytiker-upside over 20 %</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P13" t="n">
@@ -1409,33 +1417,33 @@
         <v>1</v>
       </c>
       <c r="R13" t="n">
-        <v>0.3481111314561631</v>
+        <v>0.1908475313223374</v>
       </c>
       <c r="S13" t="n">
-        <v>0.1673080525416732</v>
+        <v>0.2757298821491341</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DexCom, Inc.</t>
+          <t>Datadog, Inc.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DXCM</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>68.7</v>
+        <v>71.2</v>
       </c>
       <c r="D14" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1443,28 +1451,26 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.1701360960301399</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0.365979383233586</v>
-      </c>
+        <v>0.2694953937625746</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>0.62473</v>
+        <v>0.79536</v>
       </c>
       <c r="I14" t="n">
-        <v>0.103310004</v>
+        <v>0.0018000001</v>
       </c>
       <c r="J14" t="n">
-        <v>0.06287939525827513</v>
+        <v>0.1946964476552815</v>
       </c>
       <c r="K14" t="n">
-        <v>-0.3802542664070554</v>
+        <v>-0.5810285128029753</v>
       </c>
       <c r="L14" t="n">
-        <v>0.1653614457831325</v>
+        <v>0.3350893172454384</v>
       </c>
       <c r="M14" t="n">
-        <v>32947367936</v>
+        <v>83998416896</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -1473,43 +1479,43 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
+          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>100</v>
+        <v>88.88888888888889</v>
       </c>
       <c r="Q14" t="b">
         <v>1</v>
       </c>
       <c r="R14" t="n">
-        <v>0.4013433756067564</v>
+        <v>0.2394955649418622</v>
       </c>
       <c r="S14" t="n">
-        <v>0.1277026614627323</v>
+        <v>1.191792235717045</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GE Aerospace</t>
+          <t>Eli Lilly and Company</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GE</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>68.7</v>
+        <v>71</v>
       </c>
       <c r="D15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1517,37 +1523,37 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.1631543559703441</v>
+        <v>0.3168737488062043</v>
       </c>
       <c r="G15" t="n">
-        <v>4.460320482827598</v>
+        <v>0.5171329563234539</v>
       </c>
       <c r="H15" t="n">
-        <v>0.31051</v>
+        <v>0.83399004</v>
       </c>
       <c r="I15" t="n">
-        <v>0.05065</v>
+        <v>0.20357001</v>
       </c>
       <c r="J15" t="n">
-        <v>0.09751104545577749</v>
+        <v>0.0900853497060834</v>
       </c>
       <c r="K15" t="n">
-        <v>-0.2849592063535088</v>
+        <v>-0.4721306221588754</v>
       </c>
       <c r="L15" t="n">
-        <v>0.3421929991439169</v>
+        <v>0.1908059877458426</v>
       </c>
       <c r="M15" t="n">
-        <v>382787911680</v>
+        <v>1056890945536</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P15" t="n">
@@ -1557,33 +1563,33 @@
         <v>1</v>
       </c>
       <c r="R15" t="n">
-        <v>0.2434686346707913</v>
+        <v>0.2182561529182798</v>
       </c>
       <c r="S15" t="n">
-        <v>0.2080707511550817</v>
+        <v>0.1654455488311153</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Incyte Corporation</t>
+          <t>Seagate Technology Holdings PLC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>INCY</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>68.59999999999999</v>
+        <v>71</v>
       </c>
       <c r="D16" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1591,28 +1597,26 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.1483959547833886</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0.6156160063417289</v>
-      </c>
+        <v>0.1820341908356484</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>0.55659</v>
+        <v>0.45576</v>
       </c>
       <c r="I16" t="n">
-        <v>0.16832</v>
+        <v>0.29354998</v>
       </c>
       <c r="J16" t="n">
-        <v>0.03822105885333094</v>
+        <v>0.3729386288695309</v>
       </c>
       <c r="K16" t="n">
-        <v>-0.3626614877986997</v>
+        <v>-0.8139303115310793</v>
       </c>
       <c r="L16" t="n">
-        <v>0.1053904540162976</v>
+        <v>0.4581947908636039</v>
       </c>
       <c r="M16" t="n">
-        <v>24005494784</v>
+        <v>184496521216</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -1621,43 +1625,43 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
+          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>100</v>
+        <v>88.88888888888889</v>
       </c>
       <c r="Q16" t="b">
         <v>1</v>
       </c>
       <c r="R16" t="n">
-        <v>0.254539738159683</v>
+        <v>0.06119135769116801</v>
       </c>
       <c r="S16" t="n">
-        <v>0.1824297039767804</v>
+        <v>1.009516040690849</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Hewlett Packard Enterprise Comp</t>
+          <t>Interactive Brokers Group, Inc.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>IBKR</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>68.5</v>
+        <v>69.5</v>
       </c>
       <c r="D17" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1665,71 +1669,73 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.06370170685761956</v>
-      </c>
-      <c r="G17" t="inlineStr"/>
+        <v>0.3459787421885367</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.3328887406583814</v>
+      </c>
       <c r="H17" t="n">
-        <v>0.33776</v>
+        <v>0.93036</v>
       </c>
       <c r="I17" t="n">
-        <v>0.01966</v>
+        <v>0.022839999</v>
       </c>
       <c r="J17" t="n">
-        <v>0.3048839570063695</v>
+        <v>0.2083949675509507</v>
       </c>
       <c r="K17" t="n">
-        <v>-0.6091759554140127</v>
+        <v>-0.3288170329044745</v>
       </c>
       <c r="L17" t="n">
-        <v>0.5004858683221697</v>
+        <v>0.6337718144044321</v>
       </c>
       <c r="M17" t="n">
-        <v>66527985664</v>
+        <v>149646131200</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Positivt momentum, analytiker-upside over 20 %</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q17" t="b">
         <v>1</v>
       </c>
       <c r="R17" t="n">
-        <v>0.6697998718596914</v>
+        <v>0.05028029086934649</v>
       </c>
       <c r="S17" t="n">
-        <v>1.196724689910953</v>
+        <v>0.2665621031697569</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Delta Air Lines, Inc.</t>
+          <t>Marvell Technology, Inc.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>68.09999999999999</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="D18" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1737,27 +1743,27 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.07799197884220499</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0.5492464741024845</v>
-      </c>
+        <v>0.1144958764235571</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>0.187</v>
+        <v>0.5150299699999999</v>
       </c>
       <c r="I18" t="n">
-        <v>0.04019</v>
+        <v>0.03808</v>
       </c>
       <c r="J18" t="n">
-        <v>0.1520999017359974</v>
+        <v>0.1746260058522311</v>
       </c>
       <c r="K18" t="n">
-        <v>-0.4406594606398079</v>
+        <v>-0.7190929041697147</v>
       </c>
       <c r="L18" t="n">
-        <v>0.3451642715559961</v>
-      </c>
-      <c r="M18" t="inlineStr"/>
+        <v>0.2428420651068158</v>
+      </c>
+      <c r="M18" t="n">
+        <v>196310925312</v>
+      </c>
       <c r="N18" t="inlineStr">
         <is>
           <t>High</t>
@@ -1765,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Stærk eps-vækst, positivt momentum</t>
+          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P18" t="n">
@@ -1775,33 +1781,33 @@
         <v>1</v>
       </c>
       <c r="R18" t="n">
-        <v>0.292667485740369</v>
+        <v>0.3672517932141015</v>
       </c>
       <c r="S18" t="n">
-        <v>0.3244253549655423</v>
+        <v>1.94951442905662</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Seagate Technology Holdings PLC</t>
+          <t>Axon Enterprise, Inc.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>AXON</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>66.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="D19" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1809,26 +1815,28 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>-0.07943569063297951</v>
-      </c>
-      <c r="G19" t="inlineStr"/>
+        <v>0.3278726393918761</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-0.09393302099393697</v>
+      </c>
       <c r="H19" t="n">
-        <v>0.45576</v>
+        <v>0.5952499999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>0.29354998</v>
+        <v>0.00509</v>
       </c>
       <c r="J19" t="n">
-        <v>0.3309350708733425</v>
+        <v>0.2115816885868897</v>
       </c>
       <c r="K19" t="n">
-        <v>-0.8258248501913219</v>
+        <v>-0.4062976130015237</v>
       </c>
       <c r="L19" t="n">
-        <v>0.400732759248736</v>
+        <v>0.5207554310344823</v>
       </c>
       <c r="M19" t="n">
-        <v>188650618880</v>
+        <v>46387376128</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -1837,43 +1845,43 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Høj bruttomargin, positivt momentum, analytiker-upside over 20 %</t>
+          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q19" t="b">
         <v>1</v>
       </c>
       <c r="R19" t="n">
-        <v>0.2718075367116708</v>
+        <v>0.3376045121033731</v>
       </c>
       <c r="S19" t="n">
-        <v>0.9218372800974317</v>
+        <v>0.4287752245369121</v>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>United Rentals, Inc.</t>
+          <t>KLA Corporation</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>URI</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>66.2</v>
+        <v>67.8</v>
       </c>
       <c r="D20" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1881,28 +1889,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.1140989591195885</v>
+        <v>0.09685534331651668</v>
       </c>
       <c r="G20" t="n">
-        <v>0.09200602525921697</v>
+        <v>0.1148114331133121</v>
       </c>
       <c r="H20" t="n">
-        <v>0.3848</v>
+        <v>0.6130100000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>0.08767999999999999</v>
+        <v>0.20799999</v>
       </c>
       <c r="J20" t="n">
-        <v>0.1308004158004159</v>
+        <v>0.1652710615314723</v>
       </c>
       <c r="K20" t="n">
-        <v>-0.3712900566348842</v>
+        <v>-0.5799101509262531</v>
       </c>
       <c r="L20" t="n">
-        <v>0.3522863418048418</v>
+        <v>0.2849942551746947</v>
       </c>
       <c r="M20" t="n">
-        <v>69457641472</v>
+        <v>258839986176</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -1911,7 +1919,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, positivt momentum</t>
+          <t>Høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P20" t="n">
@@ -1921,33 +1929,33 @@
         <v>1</v>
       </c>
       <c r="R20" t="n">
-        <v>0.1267389487628878</v>
+        <v>0.1249843058235034</v>
       </c>
       <c r="S20" t="n">
-        <v>0.3772174384961748</v>
+        <v>0.4922324438519448</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Datadog, Inc.</t>
+          <t>Veeva Systems Inc.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>VEEV</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>64.59999999999999</v>
+        <v>66.3</v>
       </c>
       <c r="D21" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1955,26 +1963,28 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.2694953937625746</v>
-      </c>
-      <c r="G21" t="inlineStr"/>
+        <v>0.1402968452680178</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.2194365698361114</v>
+      </c>
       <c r="H21" t="n">
-        <v>0.79906</v>
+        <v>0.75021005</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.0021600001</v>
+        <v>0.07298</v>
       </c>
       <c r="J21" t="n">
-        <v>-0.01328581871345047</v>
+        <v>0.05932594263895519</v>
       </c>
       <c r="K21" t="n">
-        <v>-0.6417763157894737</v>
+        <v>-0.3576170434329847</v>
       </c>
       <c r="L21" t="n">
-        <v>-0.02070163448943589</v>
+        <v>0.1658923804901723</v>
       </c>
       <c r="M21" t="n">
-        <v>97390706688</v>
+        <v>37438308352</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -1983,43 +1993,43 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q21" t="b">
         <v>1</v>
       </c>
       <c r="R21" t="n">
-        <v>1.02715785060585</v>
+        <v>0.3698068423221583</v>
       </c>
       <c r="S21" t="n">
-        <v>1.090575881826636</v>
+        <v>0.2535762500379706</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cisco Systems, Inc.</t>
+          <t>United Airlines Holdings, Inc.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>UAL</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>64.09999999999999</v>
+        <v>65.5</v>
       </c>
       <c r="D22" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -2027,37 +2037,37 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.03192384157728467</v>
+        <v>0.09529134601036815</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.0254656916401832</v>
+        <v>0.6599631084110487</v>
       </c>
       <c r="H22" t="n">
-        <v>0.64296997</v>
+        <v>0.31816</v>
       </c>
       <c r="I22" t="n">
-        <v>0.07337</v>
+        <v>0.03381</v>
       </c>
       <c r="J22" t="n">
-        <v>0.1240053512860348</v>
+        <v>0.2515605125038591</v>
       </c>
       <c r="K22" t="n">
-        <v>-0.4325047471085793</v>
+        <v>-0.3467119481321396</v>
       </c>
       <c r="L22" t="n">
-        <v>0.2867144282578327</v>
+        <v>0.7255605520926088</v>
       </c>
       <c r="M22" t="n">
-        <v>456654618624</v>
+        <v>42051252224</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Høj bruttomargin, positivt momentum</t>
+          <t>Stærk eps-vækst, positivt momentum, analytiker-upside over 20 %</t>
         </is>
       </c>
       <c r="P22" t="n">
@@ -2067,33 +2077,33 @@
         <v>1</v>
       </c>
       <c r="R22" t="n">
-        <v>0.2723924311141501</v>
+        <v>0.2994985107758124</v>
       </c>
       <c r="S22" t="n">
-        <v>0.4924743780154592</v>
+        <v>0.2212272790165106</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Palo Alto Networks, Inc.</t>
+          <t>Applied Materials, Inc.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>63.4</v>
+        <v>65.3</v>
       </c>
       <c r="D23" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -2101,26 +2111,28 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.1878825003317091</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
+        <v>0.03233470456886756</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.05191743203490939</v>
+      </c>
       <c r="H23" t="n">
-        <v>0.71963996</v>
+        <v>0.48956</v>
       </c>
       <c r="I23" t="n">
-        <v>0.017719999</v>
+        <v>0.14858</v>
       </c>
       <c r="J23" t="n">
-        <v>-0.03004407570650758</v>
+        <v>0.1667787587639575</v>
       </c>
       <c r="K23" t="n">
-        <v>-0.5979316106357848</v>
+        <v>-0.7134881477909263</v>
       </c>
       <c r="L23" t="n">
-        <v>-0.05024667566004999</v>
+        <v>0.2337512673200407</v>
       </c>
       <c r="M23" t="n">
-        <v>282910949376</v>
+        <v>428055298048</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -2129,43 +2141,43 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
+          <t>Høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q23" t="b">
         <v>1</v>
       </c>
       <c r="R23" t="n">
-        <v>0.8504905923425592</v>
+        <v>0.3145583294175336</v>
       </c>
       <c r="S23" t="n">
-        <v>0.8832576181584095</v>
+        <v>0.7779648791718274</v>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Garmin Ltd.</t>
+          <t>Dell Technologies Inc.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GRMN</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>63.1</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="D24" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2173,28 +2185,28 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.142358869424539</v>
+        <v>0.03534983888485344</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1945038186480894</v>
+        <v>0.388859258627138</v>
       </c>
       <c r="H24" t="n">
-        <v>0.60081</v>
+        <v>0.19212</v>
       </c>
       <c r="I24" t="n">
-        <v>0.12174</v>
+        <v>0.07004000000000001</v>
       </c>
       <c r="J24" t="n">
-        <v>-0.06858790523690772</v>
+        <v>0.108012032527492</v>
       </c>
       <c r="K24" t="n">
-        <v>-0.3874852342827143</v>
+        <v>-0.757101615355797</v>
       </c>
       <c r="L24" t="n">
-        <v>-0.1770077906681344</v>
+        <v>0.1426651724639792</v>
       </c>
       <c r="M24" t="n">
-        <v>58773741568</v>
+        <v>293200035840</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -2203,7 +2215,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
+          <t>Stærk eps-vækst, positivt momentum</t>
         </is>
       </c>
       <c r="P24" t="n">
@@ -2213,33 +2225,33 @@
         <v>1</v>
       </c>
       <c r="R24" t="n">
-        <v>0.1749672436383698</v>
+        <v>0.9738559714176462</v>
       </c>
       <c r="S24" t="n">
-        <v>0.4474088350041829</v>
+        <v>2.951175825528565</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Monster Beverage Corporation</t>
+          <t>Howmet Aerospace Inc.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>HWM</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>63.1</v>
+        <v>64.3</v>
       </c>
       <c r="D25" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -2247,28 +2259,28 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.09536818669323455</v>
+        <v>0.1337158522423005</v>
       </c>
       <c r="G25" t="n">
-        <v>0.2027507069649817</v>
+        <v>0.495146138791156</v>
       </c>
       <c r="H25" t="n">
-        <v>0.55471003</v>
+        <v>0.36032</v>
       </c>
       <c r="I25" t="n">
-        <v>0.17725</v>
+        <v>0.12815</v>
       </c>
       <c r="J25" t="n">
-        <v>0.03037199358631759</v>
+        <v>0.1363984674329501</v>
       </c>
       <c r="K25" t="n">
-        <v>-0.3742383752004276</v>
+        <v>-0.3988576699304669</v>
       </c>
       <c r="L25" t="n">
-        <v>0.08115681233933193</v>
+        <v>0.3419727830650181</v>
       </c>
       <c r="M25" t="n">
-        <v>91492663296</v>
+        <v>112414146560</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -2277,7 +2289,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Stærk eps-vækst, høj bruttomargin, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, positivt momentum</t>
         </is>
       </c>
       <c r="P25" t="n">
@@ -2287,33 +2299,33 @@
         <v>1</v>
       </c>
       <c r="R25" t="n">
-        <v>0.2505514160510702</v>
+        <v>0.0352259372142707</v>
       </c>
       <c r="S25" t="n">
-        <v>0.2041478779483716</v>
+        <v>0.3466684453814286</v>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Morgan Stanley</t>
+          <t>Garmin Ltd.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>GRMN</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>63.1</v>
+        <v>64</v>
       </c>
       <c r="D26" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -2321,71 +2333,73 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.09524171431647233</v>
+        <v>0.142358869424539</v>
       </c>
       <c r="G26" t="n">
-        <v>0.1840868065525754</v>
+        <v>0.1945038186480894</v>
       </c>
       <c r="H26" t="n">
-        <v>0.87641</v>
-      </c>
-      <c r="I26" t="inlineStr"/>
+        <v>0.60081</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.12174</v>
+      </c>
       <c r="J26" t="n">
-        <v>0.119069024286323</v>
+        <v>-0.06627520988130842</v>
       </c>
       <c r="K26" t="n">
-        <v>-0.34000852151683</v>
+        <v>-0.3995625462382193</v>
       </c>
       <c r="L26" t="n">
-        <v>0.3501942355889726</v>
+        <v>-0.165869425213331</v>
       </c>
       <c r="M26" t="n">
-        <v>332053544960</v>
+        <v>59957067776</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Stærk eps-vækst, høj bruttomargin, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q26" t="b">
         <v>1</v>
       </c>
       <c r="R26" t="n">
-        <v>0.1101228654517645</v>
+        <v>0.2908933123836939</v>
       </c>
       <c r="S26" t="n">
-        <v>0.1726314606153021</v>
+        <v>0.5776529045416638</v>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Arista Networks, Inc.</t>
+          <t>Hewlett Packard Enterprise Comp</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>62.4</v>
+        <v>63.8</v>
       </c>
       <c r="D27" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2393,28 +2407,26 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.2714652572159764</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0.3708447402164197</v>
-      </c>
+        <v>0.06370170685761956</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>0.63537</v>
+        <v>0.33776</v>
       </c>
       <c r="I27" t="n">
-        <v>0.14359</v>
+        <v>0.01966</v>
       </c>
       <c r="J27" t="n">
-        <v>0.04013375520579809</v>
+        <v>0.2318183013904549</v>
       </c>
       <c r="K27" t="n">
-        <v>-0.3806046838660825</v>
+        <v>-0.6272078166102969</v>
       </c>
       <c r="L27" t="n">
-        <v>0.1054473497228934</v>
+        <v>0.3696036548831638</v>
       </c>
       <c r="M27" t="n">
-        <v>232807825408</v>
+        <v>70474113024</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -2423,43 +2435,43 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
+          <t>Positivt momentum, analytiker-upside over 20 %</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>100</v>
+        <v>88.88888888888889</v>
       </c>
       <c r="Q27" t="b">
         <v>1</v>
       </c>
       <c r="R27" t="n">
-        <v>0.04423599729404093</v>
+        <v>0.7971617803249145</v>
       </c>
       <c r="S27" t="n">
-        <v>0.2173473745097154</v>
+        <v>1.365472550960148</v>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Western Digital Corporation</t>
+          <t>F5, Inc.</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>FFIV</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>61.4</v>
+        <v>63.3</v>
       </c>
       <c r="D28" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -2467,27 +2479,29 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>-0.2028373451127182</v>
+        <v>0.04631913174341684</v>
       </c>
       <c r="G28" t="n">
-        <v>0.02660358695900467</v>
+        <v>0.3082491584064506</v>
       </c>
       <c r="H28" t="n">
-        <v>0.45428002</v>
+        <v>0.81865996</v>
       </c>
       <c r="I28" t="n">
-        <v>0.14648</v>
+        <v>0.07976999999999999</v>
       </c>
       <c r="J28" t="n">
-        <v>0.2433139865710707</v>
+        <v>0.08962346650675856</v>
       </c>
       <c r="K28" t="n">
-        <v>-0.8612723341299647</v>
+        <v>-0.4409214701546611</v>
       </c>
       <c r="L28" t="n">
-        <v>0.2825052854122619</v>
-      </c>
-      <c r="M28" t="inlineStr"/>
+        <v>0.2032640108800362</v>
+      </c>
+      <c r="M28" t="n">
+        <v>22663899136</v>
+      </c>
       <c r="N28" t="inlineStr">
         <is>
           <t>High</t>
@@ -2495,43 +2509,43 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Høj bruttomargin, positivt momentum, analytiker-upside over 20 %</t>
+          <t>Stærk eps-vækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q28" t="b">
         <v>1</v>
       </c>
       <c r="R28" t="n">
-        <v>0.2542163342381683</v>
+        <v>0.1600197777829866</v>
       </c>
       <c r="S28" t="n">
-        <v>0.958417094494876</v>
+        <v>0.4757200088353686</v>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CrowdStrike Holdings, Inc.</t>
+          <t>Expedia Group, Inc.</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>61</v>
+        <v>63.3</v>
       </c>
       <c r="D29" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -2539,26 +2553,28 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.2900686653697968</v>
-      </c>
-      <c r="G29" t="inlineStr"/>
+        <v>0.08087962506974211</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.6534957812135467</v>
+      </c>
       <c r="H29" t="n">
-        <v>0.75136</v>
+        <v>0.90433</v>
       </c>
       <c r="I29" t="n">
-        <v>-0.0100300005</v>
+        <v>0.061079998</v>
       </c>
       <c r="J29" t="n">
-        <v>-0.0464619334452453</v>
+        <v>0.02383713145358568</v>
       </c>
       <c r="K29" t="n">
-        <v>-0.5769724498864421</v>
+        <v>-0.4034376207029742</v>
       </c>
       <c r="L29" t="n">
-        <v>-0.08052712647612513</v>
+        <v>0.05908504866762405</v>
       </c>
       <c r="M29" t="n">
-        <v>206238220288</v>
+        <v>37287608320</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -2567,24 +2583,24 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
+          <t>Stærk eps-vækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q29" t="b">
         <v>1</v>
       </c>
       <c r="R29" t="n">
-        <v>0.7127089230317583</v>
+        <v>0.2316136480683892</v>
       </c>
       <c r="S29" t="n">
-        <v>0.717061784952312</v>
+        <v>0.3489626342686869</v>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
@@ -2600,10 +2616,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>60.5</v>
+        <v>62.5</v>
       </c>
       <c r="D30" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2617,22 +2633,22 @@
         <v>-0.09938459624739093</v>
       </c>
       <c r="H30" t="n">
-        <v>0.7846</v>
+        <v>0.7800700699999999</v>
       </c>
       <c r="I30" t="n">
-        <v>0.086660005</v>
+        <v>0.084910005</v>
       </c>
       <c r="J30" t="n">
-        <v>0.05456159034433794</v>
+        <v>0.05611930065135406</v>
       </c>
       <c r="K30" t="n">
-        <v>-0.3688320908768193</v>
+        <v>-0.3904696606102159</v>
       </c>
       <c r="L30" t="n">
-        <v>0.1479307025986525</v>
+        <v>0.1437225636523264</v>
       </c>
       <c r="M30" t="n">
-        <v>16861916160</v>
+        <v>17460494336</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -2651,33 +2667,33 @@
         <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>0.430643108686364</v>
+        <v>0.4525172025700568</v>
       </c>
       <c r="S30" t="n">
-        <v>0.1608523114354838</v>
+        <v>0.3144366553078433</v>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Lam Research Corporation</t>
+          <t>Corpay, Inc.</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>CPAY</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>60</v>
+        <v>62.3</v>
       </c>
       <c r="D31" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2685,28 +2701,28 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.02285830538778799</v>
+        <v>0.097332408585459</v>
       </c>
       <c r="G31" t="n">
-        <v>0.08212873820510125</v>
+        <v>0.06564477917470324</v>
       </c>
       <c r="H31" t="n">
-        <v>0.50469</v>
+        <v>0.79941005</v>
       </c>
       <c r="I31" t="n">
-        <v>0.22840999</v>
+        <v>0.05709</v>
       </c>
       <c r="J31" t="n">
-        <v>0.2495469603883098</v>
+        <v>0.1368511732071054</v>
       </c>
       <c r="K31" t="n">
-        <v>-0.680560741319032</v>
+        <v>-0.3565429836616277</v>
       </c>
       <c r="L31" t="n">
-        <v>0.3666784538653364</v>
+        <v>0.3838279800142754</v>
       </c>
       <c r="M31" t="n">
-        <v>368638984192</v>
+        <v>25683312640</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -2715,7 +2731,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Høj bruttomargin, positivt momentum, analytiker-upside over 20 %</t>
+          <t>Høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P31" t="n">
@@ -2725,14 +2741,14 @@
         <v>1</v>
       </c>
       <c r="R31" t="n">
-        <v>0.1371535722643684</v>
+        <v>0.2851676285900451</v>
       </c>
       <c r="S31" t="n">
-        <v>0.1829702280595702</v>
+        <v>0.1729552311683769</v>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2026-08-04 06:39:46</t>
+          <t>2026-08-09 07:56:42</t>
         </is>
       </c>
     </row>

</xml_diff>